<commit_message>
Finalizando o estudo sobre BeatifulSoap
</commit_message>
<xml_diff>
--- a/books_catalog.xlsx
+++ b/books_catalog.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000070C0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,22 +417,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>availability</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>rating</t>
         </is>

</xml_diff>